<commit_message>
chore(datos): septiembre ingerido, horas enriquecidas y el etiquetado al día
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NFeDDvCkGSN88DUHoLz1pJ
</commit_message>
<xml_diff>
--- a/data/sistema/procesada/banca/banca_unida.xlsx
+++ b/data/sistema/procesada/banca/banca_unida.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1123"/>
+  <dimension ref="A1:F1164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29624,6 +29624,1072 @@
         <v>27662.51</v>
       </c>
     </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>9635e4328061fc64bc185b1417345f76</t>
+        </is>
+      </c>
+      <c r="B1124" s="1" t="n">
+        <v>46239.59791666667</v>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA A CHICHANDA LOOR BETTY FABIOLA</t>
+        </is>
+      </c>
+      <c r="D1124" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="E1124" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1124" t="n">
+        <v>27659.01</v>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>fd8346a993278ad5698e3bb72d6bf2a0</t>
+        </is>
+      </c>
+      <c r="B1125" s="1" t="n">
+        <v>46241.52013888889</v>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIA INTERNET</t>
+        </is>
+      </c>
+      <c r="D1125" t="n">
+        <v>-10</v>
+      </c>
+      <c r="E1125" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1125" t="n">
+        <v>27649.01</v>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>4765fce891a5aee6ca867120020387b2</t>
+        </is>
+      </c>
+      <c r="B1126" s="1" t="n">
+        <v>46241.59097222222</v>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIA INTERNET</t>
+        </is>
+      </c>
+      <c r="D1126" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="E1126" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1126" t="n">
+        <v>27645.51</v>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>e4592d9a17a01eacd62cb27eb7948bf8</t>
+        </is>
+      </c>
+      <c r="B1127" s="1" t="n">
+        <v>46241.59166666667</v>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIA INTERNET</t>
+        </is>
+      </c>
+      <c r="D1127" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="E1127" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1127" t="n">
+        <v>27645.01</v>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>d45078e32dc940d832b99c69c7922253</t>
+        </is>
+      </c>
+      <c r="B1128" s="1" t="n">
+        <v>46241.76319444444</v>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIA INTERNET</t>
+        </is>
+      </c>
+      <c r="D1128" t="n">
+        <v>-27.61</v>
+      </c>
+      <c r="E1128" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1128" t="n">
+        <v>27617.4</v>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>851fffbf9e91a2a6197524858bcdff25</t>
+        </is>
+      </c>
+      <c r="B1129" s="1" t="n">
+        <v>46245.58194444444</v>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIA INTERNET</t>
+        </is>
+      </c>
+      <c r="D1129" t="n">
+        <v>-4</v>
+      </c>
+      <c r="E1129" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1129" t="n">
+        <v>27613.4</v>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>b4ee964a27ae21b9be3ab983eb009631</t>
+        </is>
+      </c>
+      <c r="B1130" s="1" t="n">
+        <v>46245.58263888889</v>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIA INTERNET</t>
+        </is>
+      </c>
+      <c r="D1130" t="n">
+        <v>-2</v>
+      </c>
+      <c r="E1130" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1130" t="n">
+        <v>27611.4</v>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>13592fadfd5d92dbd1f1cf619fea46cd</t>
+        </is>
+      </c>
+      <c r="B1131" s="1" t="n">
+        <v>46245.78680555556</v>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIA INTERNET</t>
+        </is>
+      </c>
+      <c r="D1131" t="n">
+        <v>-1.83</v>
+      </c>
+      <c r="E1131" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1131" t="n">
+        <v>27609.57</v>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>2c2fa189216602fd670dd60d3219e339</t>
+        </is>
+      </c>
+      <c r="B1132" s="1" t="n">
+        <v>46246.58263888889</v>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA A CHICHANDA LOOR BETTY FABIOLA</t>
+        </is>
+      </c>
+      <c r="D1132" t="n">
+        <v>-4</v>
+      </c>
+      <c r="E1132" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1132" t="n">
+        <v>27605.57</v>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>8cf822e91b5dc785e89ba2641b4ddaaf</t>
+        </is>
+      </c>
+      <c r="B1133" s="1" t="n">
+        <v>46248.08819444444</v>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>17056306-MASTERCARD BP  -8E-223067000075</t>
+        </is>
+      </c>
+      <c r="D1133" t="n">
+        <v>-496.85</v>
+      </c>
+      <c r="E1133" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1133" t="n">
+        <v>27108.72</v>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>9fa9f58b9d516761b1db07221dc03c3e</t>
+        </is>
+      </c>
+      <c r="B1134" s="1" t="n">
+        <v>46248.53194444445</v>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIA INTERNET</t>
+        </is>
+      </c>
+      <c r="D1134" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="E1134" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1134" t="n">
+        <v>27105.22</v>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>6b5818f01881443bc9e1b00cb56571e6</t>
+        </is>
+      </c>
+      <c r="B1135" s="1" t="n">
+        <v>46251.58125</v>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA A DAVILA IZQUIERDO MARIA DE LOURDES</t>
+        </is>
+      </c>
+      <c r="D1135" t="n">
+        <v>-8</v>
+      </c>
+      <c r="E1135" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1135" t="n">
+        <v>27097.22</v>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>d02c00c9d87e4d27ccef83cdda6449a9</t>
+        </is>
+      </c>
+      <c r="B1136" s="1" t="n">
+        <v>46251.38888888889</v>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA DE CHICAIZA NAVARRETE ALEJANDRO MANUEL</t>
+        </is>
+      </c>
+      <c r="D1136" t="n">
+        <v>6</v>
+      </c>
+      <c r="E1136" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1136" t="n">
+        <v>27103.22</v>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>9ee0259961617e323767d25ecbbd6838</t>
+        </is>
+      </c>
+      <c r="B1137" s="1" t="n">
+        <v>46251.58680555555</v>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA A QUIÑONEZ ANGULO LIGIA NELLY</t>
+        </is>
+      </c>
+      <c r="D1137" t="n">
+        <v>-30</v>
+      </c>
+      <c r="E1137" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1137" t="n">
+        <v>27073.22</v>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>883e7e3a881164b2888ace7158180ab5</t>
+        </is>
+      </c>
+      <c r="B1138" s="1" t="n">
+        <v>46251.53055555555</v>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA A QUIÑONEZ ANGULO NANCY MIRELLA</t>
+        </is>
+      </c>
+      <c r="D1138" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E1138" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1138" t="n">
+        <v>27072.22</v>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>4e5d8a38302242c5aa96c9a277cc1e62</t>
+        </is>
+      </c>
+      <c r="B1139" s="1" t="n">
+        <v>46251.7375</v>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIA INTERBANCARIA ENVIADA</t>
+        </is>
+      </c>
+      <c r="D1139" t="n">
+        <v>-6.35</v>
+      </c>
+      <c r="E1139" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1139" t="n">
+        <v>27065.87</v>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>57dd25d008415df3ffc69431fe5c6029</t>
+        </is>
+      </c>
+      <c r="B1140" s="1" t="n">
+        <v>46254.69861111111</v>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>DEPOSITO</t>
+        </is>
+      </c>
+      <c r="D1140" t="n">
+        <v>600</v>
+      </c>
+      <c r="E1140" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1140" t="n">
+        <v>27665.87</v>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>24dda2c74b3733fee80079964236b3fd</t>
+        </is>
+      </c>
+      <c r="B1141" s="1" t="n">
+        <v>46254.76527777778</v>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIA INTERBANCARIA ENVIADA</t>
+        </is>
+      </c>
+      <c r="D1141" t="n">
+        <v>-21.73</v>
+      </c>
+      <c r="E1141" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1141" t="n">
+        <v>27644.14</v>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>80b1ece640c46d73698b91d70f88fcf7</t>
+        </is>
+      </c>
+      <c r="B1142" s="1" t="n">
+        <v>46254.79305555556</v>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA A PAZMIÑO VALLEJO NORMA ISABEL</t>
+        </is>
+      </c>
+      <c r="D1142" t="n">
+        <v>-11.5</v>
+      </c>
+      <c r="E1142" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1142" t="n">
+        <v>27632.64</v>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>4e662766a5d39048c73d87f8c391125b</t>
+        </is>
+      </c>
+      <c r="B1143" s="1" t="n">
+        <v>46254.80625</v>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIA INTERBANCARIA ENVIADA</t>
+        </is>
+      </c>
+      <c r="D1143" t="n">
+        <v>-5.25</v>
+      </c>
+      <c r="E1143" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1143" t="n">
+        <v>27627.39</v>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>34f5e2da39bc4748a90f70f7a19495f2</t>
+        </is>
+      </c>
+      <c r="B1144" s="1" t="n">
+        <v>46254.80694444444</v>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>TRANSFERENCIA INTERBANCARIA ENVIADA</t>
+        </is>
+      </c>
+      <c r="D1144" t="n">
+        <v>-0.75</v>
+      </c>
+      <c r="E1144" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1144" t="n">
+        <v>27626.64</v>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>ebc9ab0f952b922bd3e9eb2b56f12acb</t>
+        </is>
+      </c>
+      <c r="B1145" s="1" t="n">
+        <v>46255.89444444444</v>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA A VERKADE MONTIEL DOMINIQUE LOURDES</t>
+        </is>
+      </c>
+      <c r="D1145" t="n">
+        <v>-496.83</v>
+      </c>
+      <c r="E1145" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1145" t="n">
+        <v>27129.81</v>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>99178caa884b1e3e643aada7b03755ed</t>
+        </is>
+      </c>
+      <c r="B1146" s="1" t="n">
+        <v>46255.89583333334</v>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA A MEDINA AYALA VIOLETA ALEJANDRA</t>
+        </is>
+      </c>
+      <c r="D1146" t="n">
+        <v>-120.04</v>
+      </c>
+      <c r="E1146" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1146" t="n">
+        <v>27009.77</v>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>eca706569c3701a2c829e41b423e8fb8</t>
+        </is>
+      </c>
+      <c r="B1147" s="1" t="n">
+        <v>46258.425</v>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>COMISION TRANSFERENCIA INTERBANCARIA ENVIADA</t>
+        </is>
+      </c>
+      <c r="D1147" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="E1147" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1147" t="n">
+        <v>27009.41</v>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>8afd8a9ff7c7e5bd43d8e182a8017475</t>
+        </is>
+      </c>
+      <c r="B1148" s="1" t="n">
+        <v>46258.425</v>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>IVA COBRADO</t>
+        </is>
+      </c>
+      <c r="D1148" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="E1148" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1148" t="n">
+        <v>27009.36</v>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>a58c03ee58fd01d5aac381b57eb1488c</t>
+        </is>
+      </c>
+      <c r="B1149" s="1" t="n">
+        <v>46258.425</v>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>TRANSF. INTERBANCARIA A ARCENTALES ARCINIEGA ANDRE SEBASTIA</t>
+        </is>
+      </c>
+      <c r="D1149" t="n">
+        <v>-10</v>
+      </c>
+      <c r="E1149" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1149" t="n">
+        <v>26999.36</v>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>9305451e69ce9ced56b8b8893c3dad5d</t>
+        </is>
+      </c>
+      <c r="B1150" s="1" t="n">
+        <v>46258.73194444444</v>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>TRANSF. DEUNA A HERNAN DARIO RAMOS VILLARREAL</t>
+        </is>
+      </c>
+      <c r="D1150" t="n">
+        <v>-10</v>
+      </c>
+      <c r="E1150" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1150" t="n">
+        <v>26989.36</v>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>ee99f8b025888c58d4a7c7307e164280</t>
+        </is>
+      </c>
+      <c r="B1151" s="1" t="n">
+        <v>46258.89236111111</v>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA DE VERKADE MONTIEL DOMINIQUE LOURDES</t>
+        </is>
+      </c>
+      <c r="D1151" t="n">
+        <v>208.67</v>
+      </c>
+      <c r="E1151" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1151" t="n">
+        <v>27198.03</v>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>1e1665cdcab2c990c8692d58173811d7</t>
+        </is>
+      </c>
+      <c r="B1152" s="1" t="n">
+        <v>46258.38541666666</v>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>CERTIFICADO DE DEPOSITO</t>
+        </is>
+      </c>
+      <c r="D1152" t="n">
+        <v>-26000</v>
+      </c>
+      <c r="E1152" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1152" t="n">
+        <v>1198.03</v>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>676d32e314370f76b33d6daae302efd3</t>
+        </is>
+      </c>
+      <c r="B1153" s="1" t="n">
+        <v>46258.39236111111</v>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA DE ARCENTALES ARCINIEGA ARIANNA NICOLE</t>
+        </is>
+      </c>
+      <c r="D1153" t="n">
+        <v>100</v>
+      </c>
+      <c r="E1153" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1153" t="n">
+        <v>1298.03</v>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>284202fd538d08c3cc3ee9b47506ea0c</t>
+        </is>
+      </c>
+      <c r="B1154" s="1" t="n">
+        <v>46258.7</v>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA DE VERKADE MONTIEL DOMINIQUE LOURDES</t>
+        </is>
+      </c>
+      <c r="D1154" t="n">
+        <v>15.06</v>
+      </c>
+      <c r="E1154" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1154" t="n">
+        <v>1313.09</v>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>2cc31b5d1f1d9c9eb529d9497a11cf6e</t>
+        </is>
+      </c>
+      <c r="B1155" s="1" t="n">
+        <v>46259.60694444444</v>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA DE VERKADE MONTIEL DOMINIQUE LOURDES</t>
+        </is>
+      </c>
+      <c r="D1155" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="E1155" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1155" t="n">
+        <v>1314.71</v>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>479a94a4d9cf8de8a24f7bf19621e723</t>
+        </is>
+      </c>
+      <c r="B1156" s="1" t="n">
+        <v>46259.60763888889</v>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA DE MEDINA AYALA VIOLETA ALEJANDRA</t>
+        </is>
+      </c>
+      <c r="D1156" t="n">
+        <v>9.35</v>
+      </c>
+      <c r="E1156" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1156" t="n">
+        <v>1324.06</v>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>7d2d0c5cacc66c51064a7760d11d2b93</t>
+        </is>
+      </c>
+      <c r="B1157" s="1" t="n">
+        <v>46259.79513888889</v>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA A MEDINA AYALA VIOLETA ALEJANDRA</t>
+        </is>
+      </c>
+      <c r="D1157" t="n">
+        <v>-2.82</v>
+      </c>
+      <c r="E1157" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1157" t="n">
+        <v>1321.24</v>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>fca4e700c0ffef8913831c95b05f6d87</t>
+        </is>
+      </c>
+      <c r="B1158" s="1" t="n">
+        <v>46260.69583333333</v>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA DE MEDINA AYALA VIOLETA ALEJANDRA</t>
+        </is>
+      </c>
+      <c r="D1158" t="n">
+        <v>49.68</v>
+      </c>
+      <c r="E1158" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1158" t="n">
+        <v>1370.92</v>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>0502398541604ed9773fb6f697442978</t>
+        </is>
+      </c>
+      <c r="B1159" s="1" t="n">
+        <v>46262.76944444444</v>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA DE MEDINA AYALA VIOLETA ALEJANDRA</t>
+        </is>
+      </c>
+      <c r="D1159" t="n">
+        <v>51.64</v>
+      </c>
+      <c r="E1159" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1159" t="n">
+        <v>1422.56</v>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>ab868890b556b432049dca857e64c98b</t>
+        </is>
+      </c>
+      <c r="B1160" s="1" t="n">
+        <v>46262.77222222222</v>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA DE VERKADE MONTIEL DOMINIQUE LOURDES</t>
+        </is>
+      </c>
+      <c r="D1160" t="n">
+        <v>43.87</v>
+      </c>
+      <c r="E1160" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1160" t="n">
+        <v>1466.43</v>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>5e8fd2a9be9399cc70dabf2b51d62f4c</t>
+        </is>
+      </c>
+      <c r="B1161" s="1" t="n">
+        <v>46262.77291666667</v>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA DE MEDINA AYALA VIOLETA ALEJANDRA</t>
+        </is>
+      </c>
+      <c r="D1161" t="n">
+        <v>6.22</v>
+      </c>
+      <c r="E1161" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1161" t="n">
+        <v>1472.65</v>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>0f3dd315c4d8bcb1a81f561e3d4bec93</t>
+        </is>
+      </c>
+      <c r="B1162" s="1" t="n">
+        <v>46262.775</v>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA DE MEDINA AYALA VIOLETA ALEJANDRA</t>
+        </is>
+      </c>
+      <c r="D1162" t="n">
+        <v>49.68</v>
+      </c>
+      <c r="E1162" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1162" t="n">
+        <v>1522.33</v>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>c1c3570ba3722857d5d5862530343218</t>
+        </is>
+      </c>
+      <c r="B1163" s="1" t="n">
+        <v>46265.03125</v>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>INTERES A SU FAVOR</t>
+        </is>
+      </c>
+      <c r="D1163" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E1163" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1163" t="n">
+        <v>1522.49</v>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>1afa6fa8c14f7948bdbc77263f6881f4</t>
+        </is>
+      </c>
+      <c r="B1164" s="1" t="n">
+        <v>46267.14375</v>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>TRANSF. DIRECTA A MEDINA AYALA VIOLETA ALEJANDRA</t>
+        </is>
+      </c>
+      <c r="D1164" t="n">
+        <v>-28.44</v>
+      </c>
+      <c r="E1164" t="inlineStr">
+        <is>
+          <t>BANCO</t>
+        </is>
+      </c>
+      <c r="F1164" t="n">
+        <v>1494.05</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>